<commit_message>
Apply 2026-09-18 expense answers to the Tax Turbo workbook.
March Home Depot goes to 524 repairs (50/50 units). Remaining Prime HD/Lowe's/IKEA split 1/3 524, 1/3 personal, 1/3 Grove. Park Chicago and Field Museum $53 to EPGC Travel; Frame Up/LAMA/Hindman parked as inventory. ComEd kept yellow with a Megan reminder.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_parts/524 Ferdinand Ave Unit 2.xlsx
+++ b/.cursor/scratch/tax_turbo_parts/524 Ferdinand Ave Unit 2.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,37 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +70,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,8 +445,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O30"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -434,67 +469,67 @@
           <t>INCOME</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>JAN</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>SEPT</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="1" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="1" t="inlineStr">
         <is>
           <t>2025 YR TOTAL</t>
         </is>
@@ -521,22 +556,22 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="2" t="n">
         <v>3479.6</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="2" t="n">
         <v>3180.81</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="2" t="n">
         <v>1757.5</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="2" t="n">
         <v>2690.16</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="2" t="n">
         <v>1261.64</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="2" t="n">
         <v>1509.84</v>
       </c>
       <c r="N3" t="n">
@@ -653,73 +688,74 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
           <t>EXPENSES</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>JAN</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="1" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="1" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="1" t="inlineStr">
         <is>
           <t>SEPT</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="1" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" s="1" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="1" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="1" t="inlineStr">
         <is>
           <t>2025 YR TOTAL</t>
         </is>
@@ -731,40 +767,40 @@
           <t>MARKETING / ADVERTISING</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O8">
@@ -778,40 +814,40 @@
           <t>SERVICE FEES</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
+      <c r="C9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O9">
@@ -825,40 +861,40 @@
           <t>REMITTED TAX</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
+      <c r="C10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O10">
@@ -872,40 +908,40 @@
           <t>INSURANCE</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>145.25</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>151.38</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>151.38</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>151.38</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>151.38</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>151.38</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>154.13</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O11">
@@ -919,40 +955,40 @@
           <t>INTERIOR MAINTENANCE</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" t="n">
+      <c r="C12" s="5" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>52.78</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>131.4</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="N12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O12">
@@ -966,40 +1002,40 @@
           <t>EXTERIOR REPAIRS</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>66.56999999999999</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>761.72</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>100.53</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>445.2</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>211.01</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>77.48999999999999</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>283.87</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>137.19</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>32.33</v>
+      </c>
+      <c r="N13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O13">
@@ -1013,40 +1049,40 @@
           <t>VILLAGE WATER AND REFUSE</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>100.56</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>90.68000000000001</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>112.84</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>137.64</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>132.77</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O14">
@@ -1060,41 +1096,41 @@
           <t>GAS</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
+      <c r="C15" s="5" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>31.37</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>32.09</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>26.31</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>22.71</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>22.72</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>53.71</v>
       </c>
       <c r="O15">
         <f>SUM(C15:N15)</f>
@@ -1107,41 +1143,41 @@
           <t>ELECTRIC</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
+      <c r="C16" s="4" t="n">
+        <v>59.04</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>57.47</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>49.15</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>54.52</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>49.73</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>57.54</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>123.54</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>106.93</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>62.88</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>46.47</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>52.88</v>
       </c>
       <c r="O16">
         <f>SUM(C16:N16)</f>
@@ -1154,40 +1190,40 @@
           <t>INTERNET</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="n">
+      <c r="C17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="N17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O17">
@@ -1201,40 +1237,40 @@
           <t>CLEANING / TURNOVER</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
+      <c r="C18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O18">
@@ -1248,40 +1284,40 @@
           <t>SUPPLIES</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
+      <c r="C19" s="5" t="n">
+        <v>110.8</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>92.95999999999999</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>68.73</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>128.37</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>176.17</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>108.93</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O19">
@@ -1295,40 +1331,40 @@
           <t>EQUIPMENT/APPLIANCE PURCHASES</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
+      <c r="C20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>73.23999999999999</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>82.27</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O20">
@@ -1342,40 +1378,40 @@
           <t>LAND TAX</t>
         </is>
       </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="n">
+      <c r="C21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O21">
@@ -1389,40 +1425,40 @@
           <t>LOANS INTEREST (from 1098)</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" t="n">
+      <c r="C22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O22">
@@ -1436,40 +1472,40 @@
           <t>MORTGAGE (cash P+I — memo only)</t>
         </is>
       </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
+      <c r="C23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O23">
@@ -1483,40 +1519,40 @@
           <t>HOA</t>
         </is>
       </c>
-      <c r="C24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
+      <c r="C24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O24">
@@ -1530,40 +1566,40 @@
           <t>OTHER</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
+      <c r="C25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="O25">
@@ -1630,6 +1666,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
@@ -1689,13 +1726,24 @@
         <v/>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Income green = Monarch Airbnb/VRBO deposits. Year total should be reconciled to PLATFORM net $17,086.94. Yellow expenses need fill (service fees/cleaning/utilities).</t>
-        </is>
-      </c>
-    </row>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>CC answers 2026-09-18: Nicor small / Prime ATT / Grove / Schauer / yard CONFIRMED. March HD $1358.65 → 524 EXTERIOR REPAIRS 50/50 with Unit 1. Remaining Prime HD/Lowe’s/IKEA 1/3 524 (50/50), 1/3 personal, 1/3 Grove. ELECTRIC yellow — REMIND JACOB: double-check ComEd with Megan (checking ACH Jacob $829.15; any extra check?). Home Depot March read as 524 (not 534). Extra Space $360 HOLD. Not tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>